<commit_message>
Initial public release of synthetic employment income microdata
</commit_message>
<xml_diff>
--- a/input_data/Per_capita_disposable_income_by_city_2018–2020.xlsx
+++ b/input_data/Per_capita_disposable_income_by_city_2018–2020.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16780"/>
+    <workbookView windowWidth="30240" windowHeight="12920"/>
   </bookViews>
   <sheets>
     <sheet name="城镇(urban)" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="341">
   <si>
     <t>city_code</t>
   </si>
@@ -5498,8 +5498,8 @@
       </c>
     </row>
     <row r="316" spans="1:3">
-      <c r="A316">
-        <v>410900</v>
+      <c r="A316" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="B316">
         <v>31042.4</v>

</xml_diff>